<commit_message>
docs(meta): update student class name to KCPM-CQ2023/3 across all submission artifacts and regenerate PDF
</commit_message>
<xml_diff>
--- a/Test_Cases_Checklist_Test_Summary.xlsx
+++ b/Test_Cases_Checklist_Test_Summary.xlsx
@@ -1888,12 +1888,12 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Class / Cohort</t>
+          <t>Class</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Computer Science / IT (23CLC)</t>
+          <t>KCPM-CQ2023/3</t>
         </is>
       </c>
     </row>

</xml_diff>